<commit_message>
- mostly added arcpy.addmessage for troubleshooting
</commit_message>
<xml_diff>
--- a/autoast/auto_ast_V2_Cuisinart_MultiP_PdfMaps/july_22.xlsx
+++ b/autoast/auto_ast_V2_Cuisinart_MultiP_PdfMaps/july_22.xlsx
@@ -1,61 +1,145 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\spatialfiles.bcgov\work\srm\nel\Local\Geomatics\Workarea\csostad\GitHub_Repositories\ast_batch_tool\autoast\auto_ast_V2_Cuisinart_MultiP_PdfMaps\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="38400" windowHeight="17832" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="17835"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ast_config" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domains" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ast_config" sheetId="1" r:id="rId1"/>
+    <sheet name="Domains" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
+  <si>
+    <t>region</t>
+  </si>
+  <si>
+    <t>feature_layer</t>
+  </si>
+  <si>
+    <t>crown_file_number</t>
+  </si>
+  <si>
+    <t>disposition_number</t>
+  </si>
+  <si>
+    <t>parcel_number</t>
+  </si>
+  <si>
+    <t>output_directory</t>
+  </si>
+  <si>
+    <t>output_directory_same_as_input</t>
+  </si>
+  <si>
+    <t>dont_overwrite_outputs</t>
+  </si>
+  <si>
+    <t>skip_conflicts_and_constraints</t>
+  </si>
+  <si>
+    <t>suppress_map_creation</t>
+  </si>
+  <si>
+    <t>add_maps_to_current</t>
+  </si>
+  <si>
+    <t>run_as_fcbc</t>
+  </si>
+  <si>
+    <t>ast_condition</t>
+  </si>
+  <si>
+    <t>file_number</t>
+  </si>
+  <si>
+    <t>\\spatialfiles.bcgov\work\srm\nel\Local\Geomatics\Workarea\csostad\Statusing\gui test\646\646.shp</t>
+  </si>
+  <si>
+    <t>Northeast</t>
+  </si>
+  <si>
+    <t>true</t>
+  </si>
+  <si>
+    <t>Cariboo</t>
+  </si>
+  <si>
+    <t>false</t>
+  </si>
+  <si>
+    <t>Kootenay_Boundary</t>
+  </si>
+  <si>
+    <t>Skeena</t>
+  </si>
+  <si>
+    <t>South_Coast</t>
+  </si>
+  <si>
+    <t>Thompson_Okanagan</t>
+  </si>
+  <si>
+    <t>West_Coast</t>
+  </si>
+  <si>
+    <t>Omineca</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color rgb="FF000000"/>
-      <sz val="11"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color rgb="FF000000"/>
-      <sz val="11"/>
-      <u val="single"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="10"/>
-      <sz val="11"/>
-      <u val="single"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -111,139 +195,80 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2"/>
   </cellStyleXfs>
   <cellXfs count="20">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:N2" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:N2" totalsRowShown="0">
   <autoFilter ref="A1:N2"/>
   <tableColumns count="14">
     <tableColumn id="1" name="region" totalsRowLabel="Total"/>
@@ -551,119 +576,86 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
-    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="23.5546875" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
-    <col width="138.88671875" bestFit="1" customWidth="1" style="6" min="2" max="2"/>
-    <col width="17.6640625" bestFit="1" customWidth="1" style="15" min="3" max="3"/>
-    <col width="23.109375" bestFit="1" customWidth="1" style="15" min="4" max="4"/>
-    <col width="17.33203125" bestFit="1" customWidth="1" style="16" min="5" max="5"/>
-    <col width="110.44140625" bestFit="1" customWidth="1" style="6" min="6" max="6"/>
-    <col width="29.33203125" bestFit="1" customWidth="1" style="17" min="7" max="7"/>
-    <col width="26.88671875" bestFit="1" customWidth="1" style="17" min="8" max="8"/>
-    <col width="29" bestFit="1" customWidth="1" style="18" min="9" max="9"/>
-    <col width="21" bestFit="1" customWidth="1" style="18" min="10" max="10"/>
-    <col width="21.33203125" bestFit="1" customWidth="1" style="17" min="11" max="11"/>
-    <col width="13.6640625" bestFit="1" customWidth="1" style="17" min="12" max="12"/>
-    <col width="14.6640625" bestFit="1" customWidth="1" style="6" min="13" max="13"/>
-    <col width="11.5546875" bestFit="1" customWidth="1" style="6" min="14" max="14"/>
-    <col width="13.5546875" bestFit="1" customWidth="1" style="6" min="15" max="15"/>
+    <col min="1" max="1" width="23.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="138.85546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.28515625" style="16" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="110.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.28515625" style="17" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.85546875" style="17" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="29" style="18" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21" style="18" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21.28515625" style="17" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.7109375" style="17" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.5703125" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="19.5" customHeight="1" s="6">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>region</t>
-        </is>
-      </c>
-      <c r="B1" s="7" t="inlineStr">
-        <is>
-          <t>feature_layer</t>
-        </is>
-      </c>
-      <c r="C1" s="8" t="inlineStr">
-        <is>
-          <t>crown_file_number</t>
-        </is>
-      </c>
-      <c r="D1" s="8" t="inlineStr">
-        <is>
-          <t>disposition_number</t>
-        </is>
-      </c>
-      <c r="E1" s="8" t="inlineStr">
-        <is>
-          <t>parcel_number</t>
-        </is>
-      </c>
-      <c r="F1" s="7" t="inlineStr">
-        <is>
-          <t>output_directory</t>
-        </is>
-      </c>
-      <c r="G1" s="9" t="inlineStr">
-        <is>
-          <t>output_directory_same_as_input</t>
-        </is>
-      </c>
-      <c r="H1" s="9" t="inlineStr">
-        <is>
-          <t>dont_overwrite_outputs</t>
-        </is>
-      </c>
-      <c r="I1" s="10" t="inlineStr">
-        <is>
-          <t>skip_conflicts_and_constraints</t>
-        </is>
-      </c>
-      <c r="J1" s="10" t="inlineStr">
-        <is>
-          <t>suppress_map_creation</t>
-        </is>
-      </c>
-      <c r="K1" s="9" t="inlineStr">
-        <is>
-          <t>add_maps_to_current</t>
-        </is>
-      </c>
-      <c r="L1" s="9" t="inlineStr">
-        <is>
-          <t>run_as_fcbc</t>
-        </is>
-      </c>
-      <c r="M1" s="7" t="inlineStr">
-        <is>
-          <t>ast_condition</t>
-        </is>
-      </c>
-      <c r="N1" s="11" t="inlineStr">
-        <is>
-          <t>file_number</t>
-        </is>
-      </c>
-      <c r="O1" s="11" t="n"/>
-    </row>
-    <row r="2" ht="19.5" customHeight="1" s="6">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>West Coast</t>
-        </is>
-      </c>
-      <c r="B2" s="19" t="inlineStr">
-        <is>
-          <t>\\spatialfiles.bcgov\work\srm\nel\Local\Geomatics\Workarea\csostad\Statusing\gui test\646\646.shp</t>
-        </is>
-      </c>
-      <c r="C2" s="8" t="n"/>
-      <c r="D2" s="8" t="n"/>
-      <c r="E2" s="8" t="n"/>
-      <c r="F2" s="13" t="n"/>
+    <row r="1" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="11"/>
+    </row>
+    <row r="2" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="13"/>
       <c r="G2" s="9" t="b">
         <v>1</v>
       </c>
@@ -682,102 +674,77 @@
       <c r="L2" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="M2" s="7" t="inlineStr">
-        <is>
-          <t>Queued</t>
-        </is>
-      </c>
-      <c r="N2" s="14" t="n"/>
-      <c r="O2" s="11" t="n"/>
+      <c r="M2" s="7"/>
+      <c r="N2" s="14"/>
+      <c r="O2" s="11"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
+    <hyperlink ref="B2" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
-    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="27.109375" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
-    <col width="13.5546875" bestFit="1" customWidth="1" style="6" min="2" max="3"/>
+    <col min="1" max="1" width="27.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="13.5703125" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.75" customHeight="1" s="6">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Northeast</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18.75" customHeight="1" s="6">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>Cariboo</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18.75" customHeight="1" s="6">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Kootenay_Boundary</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="18.75" customHeight="1" s="6">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Skeena</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="18.75" customHeight="1" s="6">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>South_Coast</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="18.75" customHeight="1" s="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Thompson_Okanagan</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="18.75" customHeight="1" s="6">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>West_Coast</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="18.75" customHeight="1" s="6">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Omineca</t>
-        </is>
+    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
tested - seems to run but didnt let it finish
</commit_message>
<xml_diff>
--- a/autoast/auto_ast_V2_Cuisinart_MultiP_PdfMaps/july_22.xlsx
+++ b/autoast/auto_ast_V2_Cuisinart_MultiP_PdfMaps/july_22.xlsx
@@ -1,61 +1,148 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\spatialfiles.bcgov\work\srm\nel\Local\Geomatics\Workarea\csostad\GitHub_Repositories\ast_batch_tool\autoast\auto_ast_V2_Cuisinart_MultiP_PdfMaps\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="38400" windowHeight="17832" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="17730"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ast_config" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domains" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ast_config" sheetId="1" r:id="rId1"/>
+    <sheet name="Domains" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+  <si>
+    <t>region</t>
+  </si>
+  <si>
+    <t>feature_layer</t>
+  </si>
+  <si>
+    <t>crown_file_number</t>
+  </si>
+  <si>
+    <t>disposition_number</t>
+  </si>
+  <si>
+    <t>parcel_number</t>
+  </si>
+  <si>
+    <t>output_directory</t>
+  </si>
+  <si>
+    <t>output_directory_same_as_input</t>
+  </si>
+  <si>
+    <t>dont_overwrite_outputs</t>
+  </si>
+  <si>
+    <t>skip_conflicts_and_constraints</t>
+  </si>
+  <si>
+    <t>suppress_map_creation</t>
+  </si>
+  <si>
+    <t>add_maps_to_current</t>
+  </si>
+  <si>
+    <t>run_as_fcbc</t>
+  </si>
+  <si>
+    <t>ast_condition</t>
+  </si>
+  <si>
+    <t>file_number</t>
+  </si>
+  <si>
+    <t>West Coast</t>
+  </si>
+  <si>
+    <t>\\spatialfiles.bcgov\work\srm\nel\Local\Geomatics\Workarea\csostad\Statusing\gui test\646\646.shp</t>
+  </si>
+  <si>
+    <t>Northeast</t>
+  </si>
+  <si>
+    <t>true</t>
+  </si>
+  <si>
+    <t>Cariboo</t>
+  </si>
+  <si>
+    <t>false</t>
+  </si>
+  <si>
+    <t>Kootenay_Boundary</t>
+  </si>
+  <si>
+    <t>Skeena</t>
+  </si>
+  <si>
+    <t>South_Coast</t>
+  </si>
+  <si>
+    <t>Thompson_Okanagan</t>
+  </si>
+  <si>
+    <t>West_Coast</t>
+  </si>
+  <si>
+    <t>Omineca</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color rgb="FF000000"/>
-      <sz val="11"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color rgb="FF000000"/>
-      <sz val="11"/>
-      <u val="single"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="10"/>
-      <sz val="11"/>
-      <u val="single"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -111,139 +198,80 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2"/>
   </cellStyleXfs>
   <cellXfs count="20">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:N2" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:N2" totalsRowShown="0">
   <autoFilter ref="A1:N2"/>
   <tableColumns count="14">
     <tableColumn id="1" name="region" totalsRowLabel="Total"/>
@@ -551,119 +579,86 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
-    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="23.5546875" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
-    <col width="138.88671875" bestFit="1" customWidth="1" style="6" min="2" max="2"/>
-    <col width="17.6640625" bestFit="1" customWidth="1" style="15" min="3" max="3"/>
-    <col width="23.109375" bestFit="1" customWidth="1" style="15" min="4" max="4"/>
-    <col width="17.33203125" bestFit="1" customWidth="1" style="16" min="5" max="5"/>
-    <col width="110.44140625" bestFit="1" customWidth="1" style="6" min="6" max="6"/>
-    <col width="29.33203125" bestFit="1" customWidth="1" style="17" min="7" max="7"/>
-    <col width="26.88671875" bestFit="1" customWidth="1" style="17" min="8" max="8"/>
-    <col width="29" bestFit="1" customWidth="1" style="18" min="9" max="9"/>
-    <col width="21" bestFit="1" customWidth="1" style="18" min="10" max="10"/>
-    <col width="21.33203125" bestFit="1" customWidth="1" style="17" min="11" max="11"/>
-    <col width="13.6640625" bestFit="1" customWidth="1" style="17" min="12" max="12"/>
-    <col width="14.6640625" bestFit="1" customWidth="1" style="6" min="13" max="13"/>
-    <col width="11.5546875" bestFit="1" customWidth="1" style="6" min="14" max="14"/>
-    <col width="13.5546875" bestFit="1" customWidth="1" style="6" min="15" max="15"/>
+    <col min="1" max="1" width="23.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="138.85546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.28515625" style="16" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="110.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.28515625" style="17" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.85546875" style="17" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="29" style="18" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21" style="18" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21.28515625" style="17" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.7109375" style="17" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.5703125" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="19.5" customHeight="1" s="6">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>region</t>
-        </is>
-      </c>
-      <c r="B1" s="7" t="inlineStr">
-        <is>
-          <t>feature_layer</t>
-        </is>
-      </c>
-      <c r="C1" s="8" t="inlineStr">
-        <is>
-          <t>crown_file_number</t>
-        </is>
-      </c>
-      <c r="D1" s="8" t="inlineStr">
-        <is>
-          <t>disposition_number</t>
-        </is>
-      </c>
-      <c r="E1" s="8" t="inlineStr">
-        <is>
-          <t>parcel_number</t>
-        </is>
-      </c>
-      <c r="F1" s="7" t="inlineStr">
-        <is>
-          <t>output_directory</t>
-        </is>
-      </c>
-      <c r="G1" s="9" t="inlineStr">
-        <is>
-          <t>output_directory_same_as_input</t>
-        </is>
-      </c>
-      <c r="H1" s="9" t="inlineStr">
-        <is>
-          <t>dont_overwrite_outputs</t>
-        </is>
-      </c>
-      <c r="I1" s="10" t="inlineStr">
-        <is>
-          <t>skip_conflicts_and_constraints</t>
-        </is>
-      </c>
-      <c r="J1" s="10" t="inlineStr">
-        <is>
-          <t>suppress_map_creation</t>
-        </is>
-      </c>
-      <c r="K1" s="9" t="inlineStr">
-        <is>
-          <t>add_maps_to_current</t>
-        </is>
-      </c>
-      <c r="L1" s="9" t="inlineStr">
-        <is>
-          <t>run_as_fcbc</t>
-        </is>
-      </c>
-      <c r="M1" s="7" t="inlineStr">
-        <is>
-          <t>ast_condition</t>
-        </is>
-      </c>
-      <c r="N1" s="11" t="inlineStr">
-        <is>
-          <t>file_number</t>
-        </is>
-      </c>
-      <c r="O1" s="11" t="n"/>
-    </row>
-    <row r="2" ht="19.5" customHeight="1" s="6">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>West Coast</t>
-        </is>
-      </c>
-      <c r="B2" s="19" t="inlineStr">
-        <is>
-          <t>\\spatialfiles.bcgov\work\srm\nel\Local\Geomatics\Workarea\csostad\Statusing\gui test\646\646.shp</t>
-        </is>
-      </c>
-      <c r="C2" s="8" t="n"/>
-      <c r="D2" s="8" t="n"/>
-      <c r="E2" s="8" t="n"/>
-      <c r="F2" s="13" t="n"/>
+    <row r="1" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="11"/>
+    </row>
+    <row r="2" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="13"/>
       <c r="G2" s="9" t="b">
         <v>1</v>
       </c>
@@ -682,102 +677,77 @@
       <c r="L2" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="M2" s="7" t="inlineStr">
-        <is>
-          <t>Queued</t>
-        </is>
-      </c>
-      <c r="N2" s="14" t="n"/>
-      <c r="O2" s="11" t="n"/>
+      <c r="M2" s="7"/>
+      <c r="N2" s="14"/>
+      <c r="O2" s="11"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
+    <hyperlink ref="B2" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
-    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="27.109375" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
-    <col width="13.5546875" bestFit="1" customWidth="1" style="6" min="2" max="3"/>
+    <col min="1" max="1" width="27.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="13.5703125" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.75" customHeight="1" s="6">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Northeast</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18.75" customHeight="1" s="6">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>Cariboo</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18.75" customHeight="1" s="6">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Kootenay_Boundary</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="18.75" customHeight="1" s="6">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Skeena</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="18.75" customHeight="1" s="6">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>South_Coast</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="18.75" customHeight="1" s="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Thompson_Okanagan</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="18.75" customHeight="1" s="6">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>West_Coast</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="18.75" customHeight="1" s="6">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Omineca</t>
-        </is>
+    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>